<commit_message>
slight changes for digitising data
</commit_message>
<xml_diff>
--- a/data/data-dictionary.xlsx
+++ b/data/data-dictionary.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leeds365-my.sharepoint.com/personal/htzt324_leeds_ac_uk/Documents/Desktop/Nika/CongoFor1.5/Git/forestplots-manual/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="99" documentId="8_{68503D99-182B-41A8-B015-980A0B4B9D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEB9FD22-7C77-4E4E-B804-9A1B307FD6FB}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="8_{68503D99-182B-41A8-B015-980A0B4B9D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{699B183F-36F9-4A2F-BB70-1D910D564996}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Field Dictionary" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Dictionary'!$A$1:$G$43</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -431,12 +434,6 @@
     <t>Original Extra Diameter</t>
   </si>
   <si>
-    <t>For Dry Forests ONLY: measured at Extra POM. May be left blank. For more information see DryFlor Field Manual https://doi.org/10.5521/forestplots.net/2020_4</t>
-  </si>
-  <si>
-    <t>For Dry Forests ONLY: measured at Extra POMr.  In most cases Extra D will be the same as Extra D0; if different, the method of quality control will be recorded in Extra Flag4. May be left blank. For more information see DryFlor Field Manual https://doi.org/10.5521/forestplots.net/2020_4</t>
-  </si>
-  <si>
     <t>If Extra POM changed from previous census</t>
   </si>
   <si>
@@ -452,45 +449,15 @@
     <t>For Dry Forests ONLY: As originally recorded in the field: May be left blank</t>
   </si>
   <si>
-    <t>For Dry Forests ONLY: the Extra POM is usually at basal height. May be left blank. For more information see DryFlor Field Manual https://doi.org/10.5521/forestplots.net/2020_4</t>
-  </si>
-  <si>
-    <t>Options can be found here: https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf. Ensure to write 'n' for a new recruit, 'a' can only be used with 'n' or 'h', and 'c' and 'd' cannot be used together. When the stem is dead, write '0'.</t>
-  </si>
-  <si>
-    <t>Options for mode of death can be found here: https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf. When a tree is alive, write '1'. When a stem is dead, only write one option from each category of rules (for example: mrs).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Options for diameter meaurement technique can be found here: https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf </t>
-  </si>
-  <si>
-    <t>Flag4 is typically 0 when a tree is recorded normally. If the POM was changed write, 60. Otherwise, if the diameter column is at all modified, this column is used to indicate how the D value was modified. Options for post field data management https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf Required if tree is alive</t>
-  </si>
-  <si>
-    <t>For more information see Appendix 1 DryFlor Field Manual https://doi.org/10.5521/forestplots.net/2020_4</t>
-  </si>
-  <si>
     <t>Comments specific to the stem during that census</t>
   </si>
   <si>
     <t>write "1" if voucher was collected from this individual, 0 if the voucher is used as a reference, leave empty if no voucher is associated with this stem.</t>
   </si>
   <si>
-    <t>Must use one of the codes provided here: https://www.forestplots.net/upload/ManualsEnglish/CrownLianaProtocols_EN.pdf</t>
-  </si>
-  <si>
-    <t>CD1 is measured orthogonal to CD2, i.e. at a direction this is at right-angles to CD2. More information here: https://forestplots.net/upload/ManualsEnglish/Crown_measurement_protocol_LoubotaPanzou_Feldpausch_07_2020_English.pdf</t>
-  </si>
-  <si>
-    <t>CD2 is measured orthogonal to CD1, i.e. at a direction this is at right-angles to CD1. More information here: https://forestplots.net/upload/ManualsEnglish/Crown_measurement_protocol_LoubotaPanzou_Feldpausch_07_2020_English.pdf</t>
-  </si>
-  <si>
     <t>leave blank if not measured</t>
   </si>
   <si>
-    <t>Options for Flag5 listed here: https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf</t>
-  </si>
-  <si>
     <t>Record if stem is broken</t>
   </si>
   <si>
@@ -510,6 +477,42 @@
   </si>
   <si>
     <t>constructed from 3 letters representing the initials of the collector and the collection number</t>
+  </si>
+  <si>
+    <t>For Dry Forests ONLY: measured at Extra POM. May be left blank. For more information see &lt;a href="https://doi.org/10.5521/forestplots.net/2020_4"&gt;DryFlor Field Manual&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>For Dry Forests ONLY: measured at Extra POMr.  In most cases Extra D will be the same as Extra D0; if different, the method of quality control will be recorded in Extra Flag4. May be left blank. For more information see &lt;a href="https://doi.org/10.5521/forestplots.net/2020_4"&gt;DryFlor Field Manual&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>For Dry Forests ONLY: the Extra POM is usually at basal height. May be left blank. For more information see &lt;a href="https://doi.org/10.5521/forestplots.net/2020_4"&gt;DryFlor Field Manual&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Options can be found in the  &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf"&gt;RAINFOR data codes&lt;/a&gt;. Ensure to write 'n' for a new recruit, 'a' can only be used with 'n' or 'h', and 'c' and 'd' cannot be used together. When the stem is dead, write '0'.</t>
+  </si>
+  <si>
+    <t>Options for mode of death can be found in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf"&gt;RAINFOR data codes&lt;/a&gt;. When a tree is alive, write '1'. When a stem is dead, only write one option from each category of rules (for example: mrs).</t>
+  </si>
+  <si>
+    <t>Options for diameter meaurement technique can be found in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf"&gt;RAINFOR data codes&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Flag4 is typically 0 when a tree is recorded normally. If the POM was changed write, 60. Otherwise, if the diameter column is at all modified, this column is used to indicate how the D value was modified. Options for post field data management can be found in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf"&gt;RAINFOR data codes&lt;/a&gt;. Required if tree is alive</t>
+  </si>
+  <si>
+    <t>For more information see Appendix 1 &lt;a href="https://doi.org/10.5521/forestplots.net/2020_4"&gt;DryFlor Field Manual&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Must use one of the codes provided in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/CrownLianaProtocols_EN.pdf"&gt;Crown Liana Protocols&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Options for Flag5 listed in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_data_codes_EN.pdf"&gt;RAINFOR data codes&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>CD1 is measured orthogonal to CD2, i.e. at a direction this is at right-angles to CD2. More information in the &lt;a href="https://forestplots.net/upload/ManualsEnglish/Crown_measurement_protocol_LoubotaPanzou_Feldpausch_07_2020_English.pdf"&gt;Crown measurement protocol&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>CD2 is measured orthogonal to CD1, i.e. at a direction this is at right-angles to CD1. More information in the &lt;a href="https://forestplots.net/upload/ManualsEnglish/Crown_measurement_protocol_LoubotaPanzou_Feldpausch_07_2020_English.pdf"&gt;Crown measurement protocol&lt;/a&gt;</t>
   </si>
 </sst>
 </file>
@@ -875,7 +878,8 @@
   <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="7" width="25" customWidth="1"/>
+    <col min="1" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="255.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1207,7 +1211,7 @@
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F19" t="s">
         <v>53</v>
@@ -1273,7 +1277,7 @@
         <v>53</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -1293,7 +1297,7 @@
         <v>53</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -1310,13 +1314,13 @@
         <v>63</v>
       </c>
       <c r="E24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F24" t="s">
         <v>53</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -1327,7 +1331,7 @@
         <v>51</v>
       </c>
       <c r="C25" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D25" t="s">
         <v>63</v>
@@ -1336,7 +1340,7 @@
         <v>59</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
@@ -1356,7 +1360,7 @@
         <v>59</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -1373,7 +1377,7 @@
         <v>73</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -1390,7 +1394,7 @@
         <v>73</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -1410,7 +1414,7 @@
         <v>73</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -1430,7 +1434,7 @@
         <v>73</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -1450,7 +1454,7 @@
         <v>83</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -1470,7 +1474,7 @@
         <v>83</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -1487,7 +1491,7 @@
         <v>88</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -1504,7 +1508,7 @@
         <v>88</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -1521,7 +1525,7 @@
         <v>88</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -1541,7 +1545,7 @@
         <v>96</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -1561,7 +1565,7 @@
         <v>96</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -1581,7 +1585,7 @@
         <v>96</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -1601,7 +1605,7 @@
         <v>73</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -1618,13 +1622,13 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="F40" t="s">
         <v>96</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -1641,7 +1645,7 @@
         <v>49</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
@@ -1655,13 +1659,13 @@
         <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="F42" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -1669,22 +1673,28 @@
         <v>110</v>
       </c>
       <c r="C43" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D43" t="s">
         <v>13</v>
       </c>
       <c r="E43" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="F43" t="s">
         <v>111</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{bdeaeda8-c81d-45ce-863e-5232a535b7cb}" enabled="0" method="" siteId="{bdeaeda8-c81d-45ce-863e-5232a535b7cb}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
adding liana data dictionary and section headers
</commit_message>
<xml_diff>
--- a/data/data-dictionary.xlsx
+++ b/data/data-dictionary.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leeds365-my.sharepoint.com/personal/htzt324_leeds_ac_uk/Documents/Desktop/Nika/CongoFor1.5/Git/forestplots-manual/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="8_{68503D99-182B-41A8-B015-980A0B4B9D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{699B183F-36F9-4A2F-BB70-1D910D564996}"/>
+  <xr:revisionPtr revIDLastSave="241" documentId="8_{68503D99-182B-41A8-B015-980A0B4B9D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C80C2B0-5066-47DD-830A-ED9909A17B3F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-12540" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Field Dictionary" sheetId="1" r:id="rId1"/>
+    <sheet name="trees" sheetId="1" r:id="rId1"/>
+    <sheet name="lianas" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Dictionary'!$A$1:$G$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">lianas!$A$1:$G$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">trees!$A$1:$G$43</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="208">
   <si>
     <t>Column</t>
   </si>
@@ -513,6 +515,156 @@
   </si>
   <si>
     <t>CD2 is measured orthogonal to CD1, i.e. at a direction this is at right-angles to CD1. More information in the &lt;a href="https://forestplots.net/upload/ManualsEnglish/Crown_measurement_protocol_LoubotaPanzou_Feldpausch_07_2020_English.pdf"&gt;Crown measurement protocol&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Old No</t>
+  </si>
+  <si>
+    <t>D.Largo</t>
+  </si>
+  <si>
+    <t>D.Altura</t>
+  </si>
+  <si>
+    <t>D.Max</t>
+  </si>
+  <si>
+    <t>POM D.Max</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
+    <t>L.F3</t>
+  </si>
+  <si>
+    <t>L.F4</t>
+  </si>
+  <si>
+    <t>A.F3</t>
+  </si>
+  <si>
+    <t>A.F4</t>
+  </si>
+  <si>
+    <t>M.F3</t>
+  </si>
+  <si>
+    <t>M.F4</t>
+  </si>
+  <si>
+    <t>Most Affected Tree</t>
+  </si>
+  <si>
+    <t>Host trees</t>
+  </si>
+  <si>
+    <t>New tag no</t>
+  </si>
+  <si>
+    <t>Current field tag number for the stem</t>
+  </si>
+  <si>
+    <t>Previous field tag number of the stem</t>
+  </si>
+  <si>
+    <t>Only stored in the database. Never used for upload. During upload the new tag no will populate the Tag No column and the value from the Tag No will move to the Old No column</t>
+  </si>
+  <si>
+    <t>Diameter at 130cm along the stem from the principal rooting point. Integer.</t>
+  </si>
+  <si>
+    <t>Diameter measured at 130cm vertically above the ground. Integer</t>
+  </si>
+  <si>
+    <t>Diameter at the widest point on the stem within 2.5m of the ground including any deformity. Integer</t>
+  </si>
+  <si>
+    <t>Point of measurement (mm) where D.Max was measured. Integer</t>
+  </si>
+  <si>
+    <t>TreeID (assigned by ForestPlots.net) of tree most heavily affected by the liana canopy.</t>
+  </si>
+  <si>
+    <t>List of TreeIDs (assigned by ForestPlots.net) of trees covered by the liana.</t>
+  </si>
+  <si>
+    <t>A single TreeID of the associated tree</t>
+  </si>
+  <si>
+    <t>A comma-separated list of the TreeIDs of the associated trees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag4 Rainfor code for post field data management for D.Max is in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag3 Rainfor code for meaurement technique for D.Max is in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag4 Rainfor code for post field data management for D.Altura is in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag3 Rainfor code for meaurement technique for D.Altura is in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag4 Rainfor code for post field data management for D.Largo is in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag3 Rainfor code for meaurement technique for D.Largo is in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. </t>
+  </si>
+  <si>
+    <t>Unique identifier of the stem created by the ForestPlots database</t>
+  </si>
+  <si>
+    <t>Should be populated for all stems</t>
+  </si>
+  <si>
+    <t>If uploading a new plot, fill this with all tag numbers. If uploading a recensus, only fill this column with the tags of new recruits or stems that changed tag.</t>
+  </si>
+  <si>
+    <t>To successfully upload the Subspecies, the Subspecies must be in the ForestPlots database. If it is not in the ForestPlots database, contact a member of the ForestPlots team with the Subspecies name and the authority that identified the Subspecies so that the new Subspecies can be added to the database.</t>
+  </si>
+  <si>
+    <t>Use Indet indet if unknown. To successfully upload the Species, the Species must be in the ForestPlots database. If it is not in the ForestPlots database, contact a member of the ForestPlots team with the Species name and the authority that identified the Species so that the new Species can be added to the database.</t>
+  </si>
+  <si>
+    <t>To successfully upload the Variety, the Variety must be in the ForestPlots database. If it is not in the ForestPlots database, contact a member of the ForestPlots team with the Variety name and the authority that identified the Variety so that the new Variety can be added to the database.</t>
+  </si>
+  <si>
+    <t>Use Indet if unknown. To successfully upload the Family, the Family must be in the ForestPlots database. If it is not in the ForestPlots database, contact a member of the ForestPlots team with the Family name and the authority that identified the Family so that the new Family can be added to the database.</t>
+  </si>
+  <si>
+    <t>Options can be found in the  &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. Ensure to write 'n' for a new recruit, 'a' can only be used with 'n' or 'h', and 'c' and 'd' cannot be used together. When the stem is dead, write '0'.</t>
+  </si>
+  <si>
+    <t>Options for mode of death can be found in the &lt;a href="https://www.forestplots.net/upload/ManualsEnglish/RAINFOR_LianaDataCodes_EN.pdf"&gt;RAINFOR liana data codes&lt;/a&gt;. When a tree is alive, write '1'. When a stem is dead, only write one option from each category of rules (for example: mrs).</t>
+  </si>
+  <si>
+    <t>The TreeID of the associated tree can be found in the ForestPlots platform. If you do not know the TreeID, write the "Most Affected Tree = (insert tag no)" in the census notes.</t>
+  </si>
+  <si>
+    <t>The TreeID of the associated tree can be found in the ForestPlots platform. If you do not know the TreeID, write the "Host trees = (insert tag no)" in the census notes.</t>
+  </si>
+  <si>
+    <t>Flag3 Rainfor code for meaurement technique for D.Largo</t>
+  </si>
+  <si>
+    <t>Flag4 Rainfor code for meaurement technique for D.Largo</t>
+  </si>
+  <si>
+    <t>Flag3 Rainfor code for meaurement technique for D.Altura</t>
+  </si>
+  <si>
+    <t>Flag4 Rainfor code for meaurement technique for D.Altura</t>
+  </si>
+  <si>
+    <t>Flag3 Rainfor code for meaurement technique for D.Max</t>
+  </si>
+  <si>
+    <t>Flag4 Rainfor code for meaurement technique for D.Max</t>
   </si>
 </sst>
 </file>
@@ -564,13 +716,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1693,6 +1848,588 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F564276E-53A1-4385-B9A7-E2392A66B79B}">
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="21.7265625" customWidth="1"/>
+    <col min="7" max="7" width="38.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G4" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>193</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" t="s">
+        <v>39</v>
+      </c>
+      <c r="G14" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>160</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>161</v>
+      </c>
+      <c r="B18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>162</v>
+      </c>
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C20" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>164</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>171</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" t="s">
+        <v>183</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>172</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s">
+        <v>184</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>165</v>
+      </c>
+      <c r="C24" t="s">
+        <v>202</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" t="s">
+        <v>73</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>166</v>
+      </c>
+      <c r="C25" t="s">
+        <v>203</v>
+      </c>
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" t="s">
+        <v>78</v>
+      </c>
+      <c r="F25" t="s">
+        <v>73</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>167</v>
+      </c>
+      <c r="C26" t="s">
+        <v>204</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" t="s">
+        <v>78</v>
+      </c>
+      <c r="F26" t="s">
+        <v>73</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>168</v>
+      </c>
+      <c r="C27" t="s">
+        <v>205</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>78</v>
+      </c>
+      <c r="F27" t="s">
+        <v>73</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>169</v>
+      </c>
+      <c r="C28" t="s">
+        <v>206</v>
+      </c>
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" t="s">
+        <v>78</v>
+      </c>
+      <c r="F28" t="s">
+        <v>73</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29" t="s">
+        <v>207</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" t="s">
+        <v>73</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" t="s">
+        <v>78</v>
+      </c>
+      <c r="F30" t="s">
+        <v>49</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" t="s">
+        <v>109</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
+        <v>142</v>
+      </c>
+      <c r="F31" t="s">
+        <v>145</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s">
+        <v>141</v>
+      </c>
+      <c r="F32" t="s">
+        <v>111</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{bdeaeda8-c81d-45ce-863e-5232a535b7cb}" enabled="0" method="" siteId="{bdeaeda8-c81d-45ce-863e-5232a535b7cb}" removed="1"/>

</xml_diff>